<commit_message>
chore: expand (characterized) bait collection
</commit_message>
<xml_diff>
--- a/data/2ODDs/char_baits.xlsx
+++ b/data/2ODDs/char_baits.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michellealexander/projects/bait_sequence_collection/data/2ODDs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E8657DA-AC9C-E142-AD2E-2F1B0817AAC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3D18FD-1462-7943-9D74-919574D76DB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11600" yWindow="5660" windowWidth="30240" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30480" yWindow="13520" windowWidth="30240" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ingroup" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3397" uniqueCount="1395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3471" uniqueCount="1432">
   <si>
     <t>gene_family</t>
   </si>
@@ -4208,13 +4208,124 @@
   </si>
   <si>
     <t>KP979707</t>
+  </si>
+  <si>
+    <t>At3g47190</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1104/pp.20.00594</t>
+  </si>
+  <si>
+    <t>MSISESYPPAFRRVTNDENPPATPVIVQGKDINIPVIDLERLDKEILREACKEWGIFRLENHGVPLALTSRLQEISESLLSLPFEKKRELFAAVKSPLSYFWGTPALNRSGDALKRGAQASNLTMLEGFNVPLSSLSSLSKLPTSTCCDDDAQEEPKLESFRVLMEEYGKHITRIAVSLFEAIAQTLNLELSGNRRSEYLSESTGLIRVYRYPQSSEEAAREALGMEVHTDSSVISILREDESGGLEIMKGEEWFCVKPVANTLIVNLGDMMQVNKVYP</t>
+  </si>
+  <si>
+    <t>MSNSESYPPEFRPLMSEKSTETGLDRSKDIDIPVIDMEHLDMEKLREACKDWGIFHLENTGIPLTFMSQVKEITESVLSLPFEEKRTLFGVNSPLSYYWGTHTVSPSGKAVTRAPQESSGHLFEGINIPLASLSRLLALSCTDPKLESFRVVMEEYGKHVTRIIVTLFEAIIETLSLELSGDQKMGYLSESTGVIRVQRYPQCTESPGLEAHTDSSVISIINQDDVGGLEFMKDGEWFNVKPLASSFVVGLGDMMQVISDEEYKSVLHKVGKRMRKKERYSIVNFVFPDKDCMFNSTRYKPFKFSEFEAQVKLDVETHGSKVGLSRFLSNP</t>
+  </si>
+  <si>
+    <t>GA2ox10</t>
+  </si>
+  <si>
+    <t>Gibberellin 2 oxidase 9</t>
+  </si>
+  <si>
+    <t>Gibberellin 2 oxidase 10</t>
+  </si>
+  <si>
+    <t>At5g58660</t>
+  </si>
+  <si>
+    <t>GAME31</t>
+  </si>
+  <si>
+    <t>E8</t>
+  </si>
+  <si>
+    <t>MESPRVEESYDKMSELKAFDDTKAGVKGLVDSGITKVPQIFVLPPKDRAKKCETHFVFPVIDLQGIDEDPIKHKEIVDKVRDASEKWGFFQVVNHGIPTSVLDRTLQGTRQFFEQDNEVKKQYYTRDTAKKVVYTSNLDLYKSSVPAASWRDTIFCYMAPNPPSLQEFPTPCGSATAQLIDYLKTAKIPRSVAAQLIEESLIDFSKDVKKLGFTLLELLSEGLGLDRSYLKDYMDCFHLFCSCNYYPPCPQPELTMGTIQHTDIGFVTILLQDDMGGLQVLHQNHWVDVPPTPGSLVVNIGDFLQLLSNDKYLSVEHRAISNNVGSRMSITCFFGESPYQSSKLYGPITELLSEDNPPKYRATTVKDHTSYLHNRGLDGTSALSRYKI</t>
+  </si>
+  <si>
+    <t>Solyc09g089580.3.1</t>
+  </si>
+  <si>
+    <t>C-27 Hydroxylase</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1093/pcp/pcab080</t>
+  </si>
+  <si>
+    <t>steroidal_glycoalkaloid_metabolism</t>
+  </si>
+  <si>
+    <t>GAME33</t>
+  </si>
+  <si>
+    <t>GAME32</t>
+  </si>
+  <si>
+    <t>GAME34</t>
+  </si>
+  <si>
+    <t>GAME40</t>
+  </si>
+  <si>
+    <t>GLYCOALKALOID METABOLISM31</t>
+  </si>
+  <si>
+    <t>GLYCOALKALOID METABOLISM32</t>
+  </si>
+  <si>
+    <t>GLYCOALKALOID METABOLISM33</t>
+  </si>
+  <si>
+    <t>GLYCOALKALOID METABOLISM34</t>
+  </si>
+  <si>
+    <t>GLYCOALKALOID METABOLISM40</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1111/nph.18064</t>
+  </si>
+  <si>
+    <t>MASTKVKIPTIDFCNSELKPNTPQWESTKVQVFEALQEFGCFEAIYDKVPNEIIEGMFDNLKEVFDFPLSKLIEYREKPFHIYDGQIPSIPLYGSVSSADLVLPNSVETFSNTFWSHGNPNFSNVAKSYFKQLMELNEMVKRMVLESLGLNNYIDEFLNSNVFMSRFTNYKVIKGENENEAALPSHTDSTYLTIIKQNQNGLQVLYKNGEWIELNHTSPNSYIVLSADIFMAWTNDKLTSAQHRVVPTGDKDRISIQFFSFPNPDYTLNVPKELVDEEHPLMFKPFKLPEFNKYIMLGAKNGLGLKNYCGL</t>
+  </si>
+  <si>
+    <t>Solyc00g136565.1.1</t>
+  </si>
+  <si>
+    <t>MASTKVKIPTIDFSNEELKPNTPLWESTKIKLFEAFQEYGCIEAIYGENPNEIREGIFDIEKKIFEFPLETKMKNHSEIPLHIGYIGQIPHLPSYESLCIPNFLAPQSVENFANIFWPHGNPEFCNLVKSYANSLLKLDEMIKRMILENLGLEKHINELLDNFVLFRFTHYKGSLSINKDENDKYDGLGAHTDNNFLTFIAQNQVNGLQINKNGEWINASISPNSFVVLSGDSFKAWTNGRLHSPLHRVAMPRENDRLSLQFNTLSKPGHFIEAPKQLVDEKHPLLFKPYEMHGLFNYVASNPGIPNAFQAYCGV</t>
+  </si>
+  <si>
+    <t>MESPRVEESYDKMSELKAFDDTKAGVKGLVDSGITKVPQIFVLPPKDRAKKCETHFVFPVIDLQGIDEDP IKHKEIVDKVRDASEKWGFFQVVNHGIPTSVLDRTLQGTRQFFEQDNEVKKQYYTRDTAKKVVYTSNLDL YKSSVPAASWRDTIFCYMAPNPPSLQEFPTPCGESLIDFSKDVKKLGFTLLELLSEGLGLDRSYLKDYMD CFHLFCSCNYYPPCPQPELTMGTIQHTDIGFVTILLQDDMGGLQVLHQNHWVDVPPTPGSLVVNIGDFLQ LLSNDKYLSVEHRAISNNVGSRMSITCFFGESPYQSSKLYGPITELLSEDNPPKYRATTVKDHTSYLHNR GLDGTSALSRYKI</t>
+  </si>
+  <si>
+    <t>SolyGAME34</t>
+  </si>
+  <si>
+    <t>SolyGAM40</t>
+  </si>
+  <si>
+    <t>MASIKSVKVPTIDFSNYQELKPNTPLWESTKIQVFEALQEYGCFEAIYDKVSKEIREETFDMSKEIFEFPLETKVKNISEKPMHGYMGMIPQLPLYESLCIPDLLNPQSLEKFSNIFWPQGNQHFCNLIKSYSNPLVELDGMLKRMISENLGLKNHIDELLNANYFLFRFTHYKGSSIASGDENNKAAGLGGHTDGNFLTFISQNQVNGLQINKNGEWIDVIISPNSYVVLAGDSFKAWTNGRLHSPLHRVTMSGQNDRLSIQLFSLSKPGHFIQAPKELVDEEHPLLFKPFEILELFKYGTTEAGYTAPPSDLFKIYCGV</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1038/s41467-019-13211-4</t>
+  </si>
+  <si>
+    <t>SolyGAME31</t>
+  </si>
+  <si>
+    <t>Solanum chacoense</t>
+  </si>
+  <si>
+    <t>MASTKVKIPTIDFCNLELKPNTPQWESIKVQVFEALKEFGCFEAIYDKVPNEIREGMFDNLKEVFDFPLSKLIEYREKPFHIYDGQVPIIELYGSVLAADLALPNSVETFANTFWSDGNPNFSNVAKSYFKQLMELNEMVTKMVLESLGLKNYIDEILNSNVFFSRFTNYKVIKGEDENKSGLPPHTDSSYLTIIKQSQNGLQVLYKNGEWIELNNTSPNSYIVLSEDAFMAWTNDSLTSAEHRVVTTGDKDRISIQLFSLPKLEYTVKAPKELVDEDHPLLFKPFNMLEYLKYTMSGDKSGTNLKDYCRL</t>
+  </si>
+  <si>
+    <t>SochGAME32</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4269,6 +4380,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -4773,10 +4890,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N306"/>
+  <dimension ref="A1:N314"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
+    <col min="4" max="4" width="29" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="33.83203125" customWidth="1"/>
+    <col min="9" max="9" width="26" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="47.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -15034,7 +15154,246 @@
         <v>1322</v>
       </c>
     </row>
+    <row r="307" spans="1:12">
+      <c r="A307" t="s">
+        <v>14</v>
+      </c>
+      <c r="D307" t="s">
+        <v>75</v>
+      </c>
+      <c r="E307" t="s">
+        <v>100</v>
+      </c>
+      <c r="F307" t="s">
+        <v>150</v>
+      </c>
+      <c r="G307" t="s">
+        <v>944</v>
+      </c>
+      <c r="H307" t="s">
+        <v>1400</v>
+      </c>
+      <c r="I307" t="s">
+        <v>1402</v>
+      </c>
+      <c r="J307" t="s">
+        <v>81</v>
+      </c>
+      <c r="K307" t="s">
+        <v>1396</v>
+      </c>
+      <c r="L307" t="s">
+        <v>1397</v>
+      </c>
+    </row>
+    <row r="308" spans="1:12">
+      <c r="A308" t="s">
+        <v>14</v>
+      </c>
+      <c r="D308" t="s">
+        <v>75</v>
+      </c>
+      <c r="E308" t="s">
+        <v>100</v>
+      </c>
+      <c r="F308" t="s">
+        <v>150</v>
+      </c>
+      <c r="G308" t="s">
+        <v>1399</v>
+      </c>
+      <c r="H308" t="s">
+        <v>1401</v>
+      </c>
+      <c r="I308" t="s">
+        <v>1395</v>
+      </c>
+      <c r="J308" t="s">
+        <v>81</v>
+      </c>
+      <c r="K308" t="s">
+        <v>1396</v>
+      </c>
+      <c r="L308" t="s">
+        <v>1398</v>
+      </c>
+    </row>
+    <row r="309" spans="1:12">
+      <c r="A309" t="s">
+        <v>14</v>
+      </c>
+      <c r="D309" t="s">
+        <v>1409</v>
+      </c>
+      <c r="F309" t="s">
+        <v>1404</v>
+      </c>
+      <c r="G309" t="s">
+        <v>1404</v>
+      </c>
+      <c r="H309" t="s">
+        <v>1407</v>
+      </c>
+      <c r="I309" t="s">
+        <v>1406</v>
+      </c>
+      <c r="J309" t="s">
+        <v>672</v>
+      </c>
+      <c r="K309" t="s">
+        <v>1408</v>
+      </c>
+      <c r="L309" t="s">
+        <v>1405</v>
+      </c>
+    </row>
+    <row r="310" spans="1:12">
+      <c r="A310" t="s">
+        <v>14</v>
+      </c>
+      <c r="D310" t="s">
+        <v>1409</v>
+      </c>
+      <c r="F310" t="s">
+        <v>1403</v>
+      </c>
+      <c r="G310" t="s">
+        <v>1403</v>
+      </c>
+      <c r="H310" t="s">
+        <v>1414</v>
+      </c>
+      <c r="I310" t="s">
+        <v>1428</v>
+      </c>
+      <c r="J310" t="s">
+        <v>672</v>
+      </c>
+      <c r="K310" t="s">
+        <v>1427</v>
+      </c>
+      <c r="L310" t="s">
+        <v>1426</v>
+      </c>
+    </row>
+    <row r="311" spans="1:12">
+      <c r="A311" t="s">
+        <v>14</v>
+      </c>
+      <c r="D311" t="s">
+        <v>1409</v>
+      </c>
+      <c r="F311" t="s">
+        <v>1411</v>
+      </c>
+      <c r="G311" t="s">
+        <v>1411</v>
+      </c>
+      <c r="H311" t="s">
+        <v>1415</v>
+      </c>
+      <c r="I311" t="s">
+        <v>1431</v>
+      </c>
+      <c r="J311" t="s">
+        <v>1429</v>
+      </c>
+      <c r="K311" t="s">
+        <v>1427</v>
+      </c>
+      <c r="L311" t="s">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="312" spans="1:12">
+      <c r="A312" t="s">
+        <v>14</v>
+      </c>
+      <c r="D312" t="s">
+        <v>1409</v>
+      </c>
+      <c r="F312" t="s">
+        <v>1410</v>
+      </c>
+      <c r="G312" t="s">
+        <v>1410</v>
+      </c>
+      <c r="H312" t="s">
+        <v>1416</v>
+      </c>
+      <c r="I312" t="s">
+        <v>1421</v>
+      </c>
+      <c r="J312" t="s">
+        <v>672</v>
+      </c>
+      <c r="K312" t="s">
+        <v>1419</v>
+      </c>
+      <c r="L312" t="s">
+        <v>1420</v>
+      </c>
+    </row>
+    <row r="313" spans="1:12">
+      <c r="A313" t="s">
+        <v>14</v>
+      </c>
+      <c r="D313" t="s">
+        <v>1409</v>
+      </c>
+      <c r="F313" t="s">
+        <v>1412</v>
+      </c>
+      <c r="G313" t="s">
+        <v>1412</v>
+      </c>
+      <c r="H313" t="s">
+        <v>1417</v>
+      </c>
+      <c r="I313" t="s">
+        <v>1424</v>
+      </c>
+      <c r="J313" t="s">
+        <v>672</v>
+      </c>
+      <c r="K313" t="s">
+        <v>1419</v>
+      </c>
+      <c r="L313" t="s">
+        <v>1422</v>
+      </c>
+    </row>
+    <row r="314" spans="1:12">
+      <c r="A314" t="s">
+        <v>14</v>
+      </c>
+      <c r="D314" t="s">
+        <v>1409</v>
+      </c>
+      <c r="F314" t="s">
+        <v>1413</v>
+      </c>
+      <c r="G314" t="s">
+        <v>1413</v>
+      </c>
+      <c r="H314" t="s">
+        <v>1418</v>
+      </c>
+      <c r="I314" t="s">
+        <v>1425</v>
+      </c>
+      <c r="J314" t="s">
+        <v>672</v>
+      </c>
+      <c r="K314" t="s">
+        <v>1419</v>
+      </c>
+      <c r="L314" t="s">
+        <v>1423</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="9" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="K28" r:id="rId1" xr:uid="{8446D661-CF4E-2C4F-B084-251C3D1ACE8A}"/>
   </hyperlinks>

</xml_diff>